<commit_message>
Address code review: exact step-key match, single-source layout, input guards
</commit_message>
<xml_diff>
--- a/docs/video-pipeline/overlay-master.workbook.xlsx
+++ b/docs/video-pipeline/overlay-master.workbook.xlsx
@@ -963,7 +963,7 @@
         <v/>
       </c>
       <c r="BG2">
-        <f>IF(TRIM($Q$2)&lt;&gt;"",TRIM($Q$2),TRIM($R$2))</f>
+        <f>IF($Q$2="",$R$2,$Q$2)</f>
         <v/>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
         <v/>
       </c>
       <c r="BG3">
-        <f>IF(TRIM($Q$3)&lt;&gt;"",TRIM($Q$3),TRIM($R$3))</f>
+        <f>IF($Q$3="",$R$3,$Q$3)</f>
         <v/>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
         <v/>
       </c>
       <c r="BG4">
-        <f>IF(TRIM($Q$4)&lt;&gt;"",TRIM($Q$4),TRIM($R$4))</f>
+        <f>IF($Q$4="",$R$4,$Q$4)</f>
         <v/>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
         <v/>
       </c>
       <c r="BG5">
-        <f>IF(TRIM($Q$5)&lt;&gt;"",TRIM($Q$5),TRIM($R$5))</f>
+        <f>IF($Q$5="",$R$5,$Q$5)</f>
         <v/>
       </c>
     </row>
@@ -1515,7 +1515,7 @@
         <v/>
       </c>
       <c r="BG6">
-        <f>IF(TRIM($Q$6)&lt;&gt;"",TRIM($Q$6),TRIM($R$6))</f>
+        <f>IF($Q$6="",$R$6,$Q$6)</f>
         <v/>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
         <v/>
       </c>
       <c r="BG7">
-        <f>IF(TRIM($Q$7)&lt;&gt;"",TRIM($Q$7),TRIM($R$7))</f>
+        <f>IF($Q$7="",$R$7,$Q$7)</f>
         <v/>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
         <v/>
       </c>
       <c r="BG8">
-        <f>IF(TRIM($Q$8)&lt;&gt;"",TRIM($Q$8),TRIM($R$8))</f>
+        <f>IF($Q$8="",$R$8,$Q$8)</f>
         <v/>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
         <v/>
       </c>
       <c r="BG9">
-        <f>IF(TRIM($Q$9)&lt;&gt;"",TRIM($Q$9),TRIM($R$9))</f>
+        <f>IF($Q$9="",$R$9,$Q$9)</f>
         <v/>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
         <v/>
       </c>
       <c r="BG10">
-        <f>IF(TRIM($Q$10)&lt;&gt;"",TRIM($Q$10),TRIM($R$10))</f>
+        <f>IF($Q$10="",$R$10,$Q$10)</f>
         <v/>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
         <v/>
       </c>
       <c r="BG11">
-        <f>IF(TRIM($Q$11)&lt;&gt;"",TRIM($Q$11),TRIM($R$11))</f>
+        <f>IF($Q$11="",$R$11,$Q$11)</f>
         <v/>
       </c>
     </row>
@@ -2343,7 +2343,7 @@
         <v/>
       </c>
       <c r="BG12">
-        <f>IF(TRIM($Q$12)&lt;&gt;"",TRIM($Q$12),TRIM($R$12))</f>
+        <f>IF($Q$12="",$R$12,$Q$12)</f>
         <v/>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
         <v/>
       </c>
       <c r="BG13">
-        <f>IF(TRIM($Q$13)&lt;&gt;"",TRIM($Q$13),TRIM($R$13))</f>
+        <f>IF($Q$13="",$R$13,$Q$13)</f>
         <v/>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
         <v/>
       </c>
       <c r="BG14">
-        <f>IF(TRIM($Q$14)&lt;&gt;"",TRIM($Q$14),TRIM($R$14))</f>
+        <f>IF($Q$14="",$R$14,$Q$14)</f>
         <v/>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
         <v/>
       </c>
       <c r="BG15">
-        <f>IF(TRIM($Q$15)&lt;&gt;"",TRIM($Q$15),TRIM($R$15))</f>
+        <f>IF($Q$15="",$R$15,$Q$15)</f>
         <v/>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
         <v/>
       </c>
       <c r="BG16">
-        <f>IF(TRIM($Q$16)&lt;&gt;"",TRIM($Q$16),TRIM($R$16))</f>
+        <f>IF($Q$16="",$R$16,$Q$16)</f>
         <v/>
       </c>
     </row>
@@ -3033,7 +3033,7 @@
         <v/>
       </c>
       <c r="BG17">
-        <f>IF(TRIM($Q$17)&lt;&gt;"",TRIM($Q$17),TRIM($R$17))</f>
+        <f>IF($Q$17="",$R$17,$Q$17)</f>
         <v/>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
         <v/>
       </c>
       <c r="BG18">
-        <f>IF(TRIM($Q$18)&lt;&gt;"",TRIM($Q$18),TRIM($R$18))</f>
+        <f>IF($Q$18="",$R$18,$Q$18)</f>
         <v/>
       </c>
     </row>
@@ -3309,7 +3309,7 @@
         <v/>
       </c>
       <c r="BG19">
-        <f>IF(TRIM($Q$19)&lt;&gt;"",TRIM($Q$19),TRIM($R$19))</f>
+        <f>IF($Q$19="",$R$19,$Q$19)</f>
         <v/>
       </c>
     </row>
@@ -3447,7 +3447,7 @@
         <v/>
       </c>
       <c r="BG20">
-        <f>IF(TRIM($Q$20)&lt;&gt;"",TRIM($Q$20),TRIM($R$20))</f>
+        <f>IF($Q$20="",$R$20,$Q$20)</f>
         <v/>
       </c>
     </row>
@@ -3585,7 +3585,7 @@
         <v/>
       </c>
       <c r="BG21">
-        <f>IF(TRIM($Q$21)&lt;&gt;"",TRIM($Q$21),TRIM($R$21))</f>
+        <f>IF($Q$21="",$R$21,$Q$21)</f>
         <v/>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
         <v/>
       </c>
       <c r="BG22">
-        <f>IF(TRIM($Q$22)&lt;&gt;"",TRIM($Q$22),TRIM($R$22))</f>
+        <f>IF($Q$22="",$R$22,$Q$22)</f>
         <v/>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
         <v/>
       </c>
       <c r="BG23">
-        <f>IF(TRIM($Q$23)&lt;&gt;"",TRIM($Q$23),TRIM($R$23))</f>
+        <f>IF($Q$23="",$R$23,$Q$23)</f>
         <v/>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
         <v/>
       </c>
       <c r="BG24">
-        <f>IF(TRIM($Q$24)&lt;&gt;"",TRIM($Q$24),TRIM($R$24))</f>
+        <f>IF($Q$24="",$R$24,$Q$24)</f>
         <v/>
       </c>
     </row>
@@ -4137,7 +4137,7 @@
         <v/>
       </c>
       <c r="BG25">
-        <f>IF(TRIM($Q$25)&lt;&gt;"",TRIM($Q$25),TRIM($R$25))</f>
+        <f>IF($Q$25="",$R$25,$Q$25)</f>
         <v/>
       </c>
     </row>
@@ -4275,7 +4275,7 @@
         <v/>
       </c>
       <c r="BG26">
-        <f>IF(TRIM($Q$26)&lt;&gt;"",TRIM($Q$26),TRIM($R$26))</f>
+        <f>IF($Q$26="",$R$26,$Q$26)</f>
         <v/>
       </c>
     </row>
@@ -4413,7 +4413,7 @@
         <v/>
       </c>
       <c r="BG27">
-        <f>IF(TRIM($Q$27)&lt;&gt;"",TRIM($Q$27),TRIM($R$27))</f>
+        <f>IF($Q$27="",$R$27,$Q$27)</f>
         <v/>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
         <v/>
       </c>
       <c r="BG28">
-        <f>IF(TRIM($Q$28)&lt;&gt;"",TRIM($Q$28),TRIM($R$28))</f>
+        <f>IF($Q$28="",$R$28,$Q$28)</f>
         <v/>
       </c>
     </row>
@@ -4689,7 +4689,7 @@
         <v/>
       </c>
       <c r="BG29">
-        <f>IF(TRIM($Q$29)&lt;&gt;"",TRIM($Q$29),TRIM($R$29))</f>
+        <f>IF($Q$29="",$R$29,$Q$29)</f>
         <v/>
       </c>
     </row>
@@ -4827,7 +4827,7 @@
         <v/>
       </c>
       <c r="BG30">
-        <f>IF(TRIM($Q$30)&lt;&gt;"",TRIM($Q$30),TRIM($R$30))</f>
+        <f>IF($Q$30="",$R$30,$Q$30)</f>
         <v/>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
         <v/>
       </c>
       <c r="BG31">
-        <f>IF(TRIM($Q$31)&lt;&gt;"",TRIM($Q$31),TRIM($R$31))</f>
+        <f>IF($Q$31="",$R$31,$Q$31)</f>
         <v/>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
         <v/>
       </c>
       <c r="BG32">
-        <f>IF(TRIM($Q$32)&lt;&gt;"",TRIM($Q$32),TRIM($R$32))</f>
+        <f>IF($Q$32="",$R$32,$Q$32)</f>
         <v/>
       </c>
     </row>
@@ -5241,7 +5241,7 @@
         <v/>
       </c>
       <c r="BG33">
-        <f>IF(TRIM($Q$33)&lt;&gt;"",TRIM($Q$33),TRIM($R$33))</f>
+        <f>IF($Q$33="",$R$33,$Q$33)</f>
         <v/>
       </c>
     </row>
@@ -5379,7 +5379,7 @@
         <v/>
       </c>
       <c r="BG34">
-        <f>IF(TRIM($Q$34)&lt;&gt;"",TRIM($Q$34),TRIM($R$34))</f>
+        <f>IF($Q$34="",$R$34,$Q$34)</f>
         <v/>
       </c>
     </row>
@@ -5517,7 +5517,7 @@
         <v/>
       </c>
       <c r="BG35">
-        <f>IF(TRIM($Q$35)&lt;&gt;"",TRIM($Q$35),TRIM($R$35))</f>
+        <f>IF($Q$35="",$R$35,$Q$35)</f>
         <v/>
       </c>
     </row>
@@ -5655,7 +5655,7 @@
         <v/>
       </c>
       <c r="BG36">
-        <f>IF(TRIM($Q$36)&lt;&gt;"",TRIM($Q$36),TRIM($R$36))</f>
+        <f>IF($Q$36="",$R$36,$Q$36)</f>
         <v/>
       </c>
     </row>
@@ -5793,7 +5793,7 @@
         <v/>
       </c>
       <c r="BG37">
-        <f>IF(TRIM($Q$37)&lt;&gt;"",TRIM($Q$37),TRIM($R$37))</f>
+        <f>IF($Q$37="",$R$37,$Q$37)</f>
         <v/>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
         <v/>
       </c>
       <c r="BG38">
-        <f>IF(TRIM($Q$38)&lt;&gt;"",TRIM($Q$38),TRIM($R$38))</f>
+        <f>IF($Q$38="",$R$38,$Q$38)</f>
         <v/>
       </c>
     </row>
@@ -6069,7 +6069,7 @@
         <v/>
       </c>
       <c r="BG39">
-        <f>IF(TRIM($Q$39)&lt;&gt;"",TRIM($Q$39),TRIM($R$39))</f>
+        <f>IF($Q$39="",$R$39,$Q$39)</f>
         <v/>
       </c>
     </row>
@@ -6207,7 +6207,7 @@
         <v/>
       </c>
       <c r="BG40">
-        <f>IF(TRIM($Q$40)&lt;&gt;"",TRIM($Q$40),TRIM($R$40))</f>
+        <f>IF($Q$40="",$R$40,$Q$40)</f>
         <v/>
       </c>
     </row>
@@ -6345,7 +6345,7 @@
         <v/>
       </c>
       <c r="BG41">
-        <f>IF(TRIM($Q$41)&lt;&gt;"",TRIM($Q$41),TRIM($R$41))</f>
+        <f>IF($Q$41="",$R$41,$Q$41)</f>
         <v/>
       </c>
     </row>
@@ -6483,7 +6483,7 @@
         <v/>
       </c>
       <c r="BG42">
-        <f>IF(TRIM($Q$42)&lt;&gt;"",TRIM($Q$42),TRIM($R$42))</f>
+        <f>IF($Q$42="",$R$42,$Q$42)</f>
         <v/>
       </c>
     </row>
@@ -6621,7 +6621,7 @@
         <v/>
       </c>
       <c r="BG43">
-        <f>IF(TRIM($Q$43)&lt;&gt;"",TRIM($Q$43),TRIM($R$43))</f>
+        <f>IF($Q$43="",$R$43,$Q$43)</f>
         <v/>
       </c>
     </row>
@@ -6759,7 +6759,7 @@
         <v/>
       </c>
       <c r="BG44">
-        <f>IF(TRIM($Q$44)&lt;&gt;"",TRIM($Q$44),TRIM($R$44))</f>
+        <f>IF($Q$44="",$R$44,$Q$44)</f>
         <v/>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
         <v/>
       </c>
       <c r="BG45">
-        <f>IF(TRIM($Q$45)&lt;&gt;"",TRIM($Q$45),TRIM($R$45))</f>
+        <f>IF($Q$45="",$R$45,$Q$45)</f>
         <v/>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
         <v/>
       </c>
       <c r="BG46">
-        <f>IF(TRIM($Q$46)&lt;&gt;"",TRIM($Q$46),TRIM($R$46))</f>
+        <f>IF($Q$46="",$R$46,$Q$46)</f>
         <v/>
       </c>
     </row>
@@ -7173,7 +7173,7 @@
         <v/>
       </c>
       <c r="BG47">
-        <f>IF(TRIM($Q$47)&lt;&gt;"",TRIM($Q$47),TRIM($R$47))</f>
+        <f>IF($Q$47="",$R$47,$Q$47)</f>
         <v/>
       </c>
     </row>
@@ -7311,7 +7311,7 @@
         <v/>
       </c>
       <c r="BG48">
-        <f>IF(TRIM($Q$48)&lt;&gt;"",TRIM($Q$48),TRIM($R$48))</f>
+        <f>IF($Q$48="",$R$48,$Q$48)</f>
         <v/>
       </c>
     </row>
@@ -7449,7 +7449,7 @@
         <v/>
       </c>
       <c r="BG49">
-        <f>IF(TRIM($Q$49)&lt;&gt;"",TRIM($Q$49),TRIM($R$49))</f>
+        <f>IF($Q$49="",$R$49,$Q$49)</f>
         <v/>
       </c>
     </row>
@@ -7587,7 +7587,7 @@
         <v/>
       </c>
       <c r="BG50">
-        <f>IF(TRIM($Q$50)&lt;&gt;"",TRIM($Q$50),TRIM($R$50))</f>
+        <f>IF($Q$50="",$R$50,$Q$50)</f>
         <v/>
       </c>
     </row>
@@ -7725,7 +7725,7 @@
         <v/>
       </c>
       <c r="BG51">
-        <f>IF(TRIM($Q$51)&lt;&gt;"",TRIM($Q$51),TRIM($R$51))</f>
+        <f>IF($Q$51="",$R$51,$Q$51)</f>
         <v/>
       </c>
     </row>
@@ -7863,7 +7863,7 @@
         <v/>
       </c>
       <c r="BG52">
-        <f>IF(TRIM($Q$52)&lt;&gt;"",TRIM($Q$52),TRIM($R$52))</f>
+        <f>IF($Q$52="",$R$52,$Q$52)</f>
         <v/>
       </c>
     </row>
@@ -8001,7 +8001,7 @@
         <v/>
       </c>
       <c r="BG53">
-        <f>IF(TRIM($Q$53)&lt;&gt;"",TRIM($Q$53),TRIM($R$53))</f>
+        <f>IF($Q$53="",$R$53,$Q$53)</f>
         <v/>
       </c>
     </row>
@@ -8139,7 +8139,7 @@
         <v/>
       </c>
       <c r="BG54">
-        <f>IF(TRIM($Q$54)&lt;&gt;"",TRIM($Q$54),TRIM($R$54))</f>
+        <f>IF($Q$54="",$R$54,$Q$54)</f>
         <v/>
       </c>
     </row>
@@ -8277,7 +8277,7 @@
         <v/>
       </c>
       <c r="BG55">
-        <f>IF(TRIM($Q$55)&lt;&gt;"",TRIM($Q$55),TRIM($R$55))</f>
+        <f>IF($Q$55="",$R$55,$Q$55)</f>
         <v/>
       </c>
     </row>
@@ -8415,7 +8415,7 @@
         <v/>
       </c>
       <c r="BG56">
-        <f>IF(TRIM($Q$56)&lt;&gt;"",TRIM($Q$56),TRIM($R$56))</f>
+        <f>IF($Q$56="",$R$56,$Q$56)</f>
         <v/>
       </c>
     </row>
@@ -8553,7 +8553,7 @@
         <v/>
       </c>
       <c r="BG57">
-        <f>IF(TRIM($Q$57)&lt;&gt;"",TRIM($Q$57),TRIM($R$57))</f>
+        <f>IF($Q$57="",$R$57,$Q$57)</f>
         <v/>
       </c>
     </row>
@@ -8691,7 +8691,7 @@
         <v/>
       </c>
       <c r="BG58">
-        <f>IF(TRIM($Q$58)&lt;&gt;"",TRIM($Q$58),TRIM($R$58))</f>
+        <f>IF($Q$58="",$R$58,$Q$58)</f>
         <v/>
       </c>
     </row>
@@ -8829,7 +8829,7 @@
         <v/>
       </c>
       <c r="BG59">
-        <f>IF(TRIM($Q$59)&lt;&gt;"",TRIM($Q$59),TRIM($R$59))</f>
+        <f>IF($Q$59="",$R$59,$Q$59)</f>
         <v/>
       </c>
     </row>
@@ -8967,7 +8967,7 @@
         <v/>
       </c>
       <c r="BG60">
-        <f>IF(TRIM($Q$60)&lt;&gt;"",TRIM($Q$60),TRIM($R$60))</f>
+        <f>IF($Q$60="",$R$60,$Q$60)</f>
         <v/>
       </c>
     </row>
@@ -9105,7 +9105,7 @@
         <v/>
       </c>
       <c r="BG61">
-        <f>IF(TRIM($Q$61)&lt;&gt;"",TRIM($Q$61),TRIM($R$61))</f>
+        <f>IF($Q$61="",$R$61,$Q$61)</f>
         <v/>
       </c>
     </row>
@@ -9243,7 +9243,7 @@
         <v/>
       </c>
       <c r="BG62">
-        <f>IF(TRIM($Q$62)&lt;&gt;"",TRIM($Q$62),TRIM($R$62))</f>
+        <f>IF($Q$62="",$R$62,$Q$62)</f>
         <v/>
       </c>
     </row>
@@ -9381,7 +9381,7 @@
         <v/>
       </c>
       <c r="BG63">
-        <f>IF(TRIM($Q$63)&lt;&gt;"",TRIM($Q$63),TRIM($R$63))</f>
+        <f>IF($Q$63="",$R$63,$Q$63)</f>
         <v/>
       </c>
     </row>
@@ -9519,7 +9519,7 @@
         <v/>
       </c>
       <c r="BG64">
-        <f>IF(TRIM($Q$64)&lt;&gt;"",TRIM($Q$64),TRIM($R$64))</f>
+        <f>IF($Q$64="",$R$64,$Q$64)</f>
         <v/>
       </c>
     </row>
@@ -9657,7 +9657,7 @@
         <v/>
       </c>
       <c r="BG65">
-        <f>IF(TRIM($Q$65)&lt;&gt;"",TRIM($Q$65),TRIM($R$65))</f>
+        <f>IF($Q$65="",$R$65,$Q$65)</f>
         <v/>
       </c>
     </row>
@@ -9795,7 +9795,7 @@
         <v/>
       </c>
       <c r="BG66">
-        <f>IF(TRIM($Q$66)&lt;&gt;"",TRIM($Q$66),TRIM($R$66))</f>
+        <f>IF($Q$66="",$R$66,$Q$66)</f>
         <v/>
       </c>
     </row>
@@ -9933,7 +9933,7 @@
         <v/>
       </c>
       <c r="BG67">
-        <f>IF(TRIM($Q$67)&lt;&gt;"",TRIM($Q$67),TRIM($R$67))</f>
+        <f>IF($Q$67="",$R$67,$Q$67)</f>
         <v/>
       </c>
     </row>
@@ -10071,7 +10071,7 @@
         <v/>
       </c>
       <c r="BG68">
-        <f>IF(TRIM($Q$68)&lt;&gt;"",TRIM($Q$68),TRIM($R$68))</f>
+        <f>IF($Q$68="",$R$68,$Q$68)</f>
         <v/>
       </c>
     </row>
@@ -10209,7 +10209,7 @@
         <v/>
       </c>
       <c r="BG69">
-        <f>IF(TRIM($Q$69)&lt;&gt;"",TRIM($Q$69),TRIM($R$69))</f>
+        <f>IF($Q$69="",$R$69,$Q$69)</f>
         <v/>
       </c>
     </row>
@@ -10347,7 +10347,7 @@
         <v/>
       </c>
       <c r="BG70">
-        <f>IF(TRIM($Q$70)&lt;&gt;"",TRIM($Q$70),TRIM($R$70))</f>
+        <f>IF($Q$70="",$R$70,$Q$70)</f>
         <v/>
       </c>
     </row>
@@ -10485,7 +10485,7 @@
         <v/>
       </c>
       <c r="BG71">
-        <f>IF(TRIM($Q$71)&lt;&gt;"",TRIM($Q$71),TRIM($R$71))</f>
+        <f>IF($Q$71="",$R$71,$Q$71)</f>
         <v/>
       </c>
     </row>
@@ -10623,7 +10623,7 @@
         <v/>
       </c>
       <c r="BG72">
-        <f>IF(TRIM($Q$72)&lt;&gt;"",TRIM($Q$72),TRIM($R$72))</f>
+        <f>IF($Q$72="",$R$72,$Q$72)</f>
         <v/>
       </c>
     </row>
@@ -10761,7 +10761,7 @@
         <v/>
       </c>
       <c r="BG73">
-        <f>IF(TRIM($Q$73)&lt;&gt;"",TRIM($Q$73),TRIM($R$73))</f>
+        <f>IF($Q$73="",$R$73,$Q$73)</f>
         <v/>
       </c>
     </row>
@@ -10899,7 +10899,7 @@
         <v/>
       </c>
       <c r="BG74">
-        <f>IF(TRIM($Q$74)&lt;&gt;"",TRIM($Q$74),TRIM($R$74))</f>
+        <f>IF($Q$74="",$R$74,$Q$74)</f>
         <v/>
       </c>
     </row>
@@ -11037,7 +11037,7 @@
         <v/>
       </c>
       <c r="BG75">
-        <f>IF(TRIM($Q$75)&lt;&gt;"",TRIM($Q$75),TRIM($R$75))</f>
+        <f>IF($Q$75="",$R$75,$Q$75)</f>
         <v/>
       </c>
     </row>
@@ -11175,7 +11175,7 @@
         <v/>
       </c>
       <c r="BG76">
-        <f>IF(TRIM($Q$76)&lt;&gt;"",TRIM($Q$76),TRIM($R$76))</f>
+        <f>IF($Q$76="",$R$76,$Q$76)</f>
         <v/>
       </c>
     </row>
@@ -11313,7 +11313,7 @@
         <v/>
       </c>
       <c r="BG77">
-        <f>IF(TRIM($Q$77)&lt;&gt;"",TRIM($Q$77),TRIM($R$77))</f>
+        <f>IF($Q$77="",$R$77,$Q$77)</f>
         <v/>
       </c>
     </row>
@@ -11451,7 +11451,7 @@
         <v/>
       </c>
       <c r="BG78">
-        <f>IF(TRIM($Q$78)&lt;&gt;"",TRIM($Q$78),TRIM($R$78))</f>
+        <f>IF($Q$78="",$R$78,$Q$78)</f>
         <v/>
       </c>
     </row>
@@ -11589,7 +11589,7 @@
         <v/>
       </c>
       <c r="BG79">
-        <f>IF(TRIM($Q$79)&lt;&gt;"",TRIM($Q$79),TRIM($R$79))</f>
+        <f>IF($Q$79="",$R$79,$Q$79)</f>
         <v/>
       </c>
     </row>
@@ -11727,7 +11727,7 @@
         <v/>
       </c>
       <c r="BG80">
-        <f>IF(TRIM($Q$80)&lt;&gt;"",TRIM($Q$80),TRIM($R$80))</f>
+        <f>IF($Q$80="",$R$80,$Q$80)</f>
         <v/>
       </c>
     </row>
@@ -11865,7 +11865,7 @@
         <v/>
       </c>
       <c r="BG81">
-        <f>IF(TRIM($Q$81)&lt;&gt;"",TRIM($Q$81),TRIM($R$81))</f>
+        <f>IF($Q$81="",$R$81,$Q$81)</f>
         <v/>
       </c>
     </row>
@@ -12003,7 +12003,7 @@
         <v/>
       </c>
       <c r="BG82">
-        <f>IF(TRIM($Q$82)&lt;&gt;"",TRIM($Q$82),TRIM($R$82))</f>
+        <f>IF($Q$82="",$R$82,$Q$82)</f>
         <v/>
       </c>
     </row>
@@ -12141,7 +12141,7 @@
         <v/>
       </c>
       <c r="BG83">
-        <f>IF(TRIM($Q$83)&lt;&gt;"",TRIM($Q$83),TRIM($R$83))</f>
+        <f>IF($Q$83="",$R$83,$Q$83)</f>
         <v/>
       </c>
     </row>
@@ -12279,7 +12279,7 @@
         <v/>
       </c>
       <c r="BG84">
-        <f>IF(TRIM($Q$84)&lt;&gt;"",TRIM($Q$84),TRIM($R$84))</f>
+        <f>IF($Q$84="",$R$84,$Q$84)</f>
         <v/>
       </c>
     </row>
@@ -12417,7 +12417,7 @@
         <v/>
       </c>
       <c r="BG85">
-        <f>IF(TRIM($Q$85)&lt;&gt;"",TRIM($Q$85),TRIM($R$85))</f>
+        <f>IF($Q$85="",$R$85,$Q$85)</f>
         <v/>
       </c>
     </row>
@@ -12555,7 +12555,7 @@
         <v/>
       </c>
       <c r="BG86">
-        <f>IF(TRIM($Q$86)&lt;&gt;"",TRIM($Q$86),TRIM($R$86))</f>
+        <f>IF($Q$86="",$R$86,$Q$86)</f>
         <v/>
       </c>
     </row>
@@ -12693,7 +12693,7 @@
         <v/>
       </c>
       <c r="BG87">
-        <f>IF(TRIM($Q$87)&lt;&gt;"",TRIM($Q$87),TRIM($R$87))</f>
+        <f>IF($Q$87="",$R$87,$Q$87)</f>
         <v/>
       </c>
     </row>
@@ -12831,7 +12831,7 @@
         <v/>
       </c>
       <c r="BG88">
-        <f>IF(TRIM($Q$88)&lt;&gt;"",TRIM($Q$88),TRIM($R$88))</f>
+        <f>IF($Q$88="",$R$88,$Q$88)</f>
         <v/>
       </c>
     </row>
@@ -12969,7 +12969,7 @@
         <v/>
       </c>
       <c r="BG89">
-        <f>IF(TRIM($Q$89)&lt;&gt;"",TRIM($Q$89),TRIM($R$89))</f>
+        <f>IF($Q$89="",$R$89,$Q$89)</f>
         <v/>
       </c>
     </row>
@@ -13107,7 +13107,7 @@
         <v/>
       </c>
       <c r="BG90">
-        <f>IF(TRIM($Q$90)&lt;&gt;"",TRIM($Q$90),TRIM($R$90))</f>
+        <f>IF($Q$90="",$R$90,$Q$90)</f>
         <v/>
       </c>
     </row>
@@ -13245,7 +13245,7 @@
         <v/>
       </c>
       <c r="BG91">
-        <f>IF(TRIM($Q$91)&lt;&gt;"",TRIM($Q$91),TRIM($R$91))</f>
+        <f>IF($Q$91="",$R$91,$Q$91)</f>
         <v/>
       </c>
     </row>
@@ -13383,7 +13383,7 @@
         <v/>
       </c>
       <c r="BG92">
-        <f>IF(TRIM($Q$92)&lt;&gt;"",TRIM($Q$92),TRIM($R$92))</f>
+        <f>IF($Q$92="",$R$92,$Q$92)</f>
         <v/>
       </c>
     </row>
@@ -13521,7 +13521,7 @@
         <v/>
       </c>
       <c r="BG93">
-        <f>IF(TRIM($Q$93)&lt;&gt;"",TRIM($Q$93),TRIM($R$93))</f>
+        <f>IF($Q$93="",$R$93,$Q$93)</f>
         <v/>
       </c>
     </row>
@@ -13659,7 +13659,7 @@
         <v/>
       </c>
       <c r="BG94">
-        <f>IF(TRIM($Q$94)&lt;&gt;"",TRIM($Q$94),TRIM($R$94))</f>
+        <f>IF($Q$94="",$R$94,$Q$94)</f>
         <v/>
       </c>
     </row>
@@ -13797,7 +13797,7 @@
         <v/>
       </c>
       <c r="BG95">
-        <f>IF(TRIM($Q$95)&lt;&gt;"",TRIM($Q$95),TRIM($R$95))</f>
+        <f>IF($Q$95="",$R$95,$Q$95)</f>
         <v/>
       </c>
     </row>
@@ -13935,7 +13935,7 @@
         <v/>
       </c>
       <c r="BG96">
-        <f>IF(TRIM($Q$96)&lt;&gt;"",TRIM($Q$96),TRIM($R$96))</f>
+        <f>IF($Q$96="",$R$96,$Q$96)</f>
         <v/>
       </c>
     </row>
@@ -14073,7 +14073,7 @@
         <v/>
       </c>
       <c r="BG97">
-        <f>IF(TRIM($Q$97)&lt;&gt;"",TRIM($Q$97),TRIM($R$97))</f>
+        <f>IF($Q$97="",$R$97,$Q$97)</f>
         <v/>
       </c>
     </row>
@@ -14211,7 +14211,7 @@
         <v/>
       </c>
       <c r="BG98">
-        <f>IF(TRIM($Q$98)&lt;&gt;"",TRIM($Q$98),TRIM($R$98))</f>
+        <f>IF($Q$98="",$R$98,$Q$98)</f>
         <v/>
       </c>
     </row>
@@ -14349,7 +14349,7 @@
         <v/>
       </c>
       <c r="BG99">
-        <f>IF(TRIM($Q$99)&lt;&gt;"",TRIM($Q$99),TRIM($R$99))</f>
+        <f>IF($Q$99="",$R$99,$Q$99)</f>
         <v/>
       </c>
     </row>
@@ -14487,7 +14487,7 @@
         <v/>
       </c>
       <c r="BG100">
-        <f>IF(TRIM($Q$100)&lt;&gt;"",TRIM($Q$100),TRIM($R$100))</f>
+        <f>IF($Q$100="",$R$100,$Q$100)</f>
         <v/>
       </c>
     </row>
@@ -14625,7 +14625,7 @@
         <v/>
       </c>
       <c r="BG101">
-        <f>IF(TRIM($Q$101)&lt;&gt;"",TRIM($Q$101),TRIM($R$101))</f>
+        <f>IF($Q$101="",$R$101,$Q$101)</f>
         <v/>
       </c>
     </row>
@@ -14763,7 +14763,7 @@
         <v/>
       </c>
       <c r="BG102">
-        <f>IF(TRIM($Q$102)&lt;&gt;"",TRIM($Q$102),TRIM($R$102))</f>
+        <f>IF($Q$102="",$R$102,$Q$102)</f>
         <v/>
       </c>
     </row>
@@ -14901,7 +14901,7 @@
         <v/>
       </c>
       <c r="BG103">
-        <f>IF(TRIM($Q$103)&lt;&gt;"",TRIM($Q$103),TRIM($R$103))</f>
+        <f>IF($Q$103="",$R$103,$Q$103)</f>
         <v/>
       </c>
     </row>
@@ -15039,7 +15039,7 @@
         <v/>
       </c>
       <c r="BG104">
-        <f>IF(TRIM($Q$104)&lt;&gt;"",TRIM($Q$104),TRIM($R$104))</f>
+        <f>IF($Q$104="",$R$104,$Q$104)</f>
         <v/>
       </c>
     </row>
@@ -15177,7 +15177,7 @@
         <v/>
       </c>
       <c r="BG105">
-        <f>IF(TRIM($Q$105)&lt;&gt;"",TRIM($Q$105),TRIM($R$105))</f>
+        <f>IF($Q$105="",$R$105,$Q$105)</f>
         <v/>
       </c>
     </row>
@@ -15315,7 +15315,7 @@
         <v/>
       </c>
       <c r="BG106">
-        <f>IF(TRIM($Q$106)&lt;&gt;"",TRIM($Q$106),TRIM($R$106))</f>
+        <f>IF($Q$106="",$R$106,$Q$106)</f>
         <v/>
       </c>
     </row>
@@ -15453,7 +15453,7 @@
         <v/>
       </c>
       <c r="BG107">
-        <f>IF(TRIM($Q$107)&lt;&gt;"",TRIM($Q$107),TRIM($R$107))</f>
+        <f>IF($Q$107="",$R$107,$Q$107)</f>
         <v/>
       </c>
     </row>
@@ -15591,7 +15591,7 @@
         <v/>
       </c>
       <c r="BG108">
-        <f>IF(TRIM($Q$108)&lt;&gt;"",TRIM($Q$108),TRIM($R$108))</f>
+        <f>IF($Q$108="",$R$108,$Q$108)</f>
         <v/>
       </c>
     </row>
@@ -15729,7 +15729,7 @@
         <v/>
       </c>
       <c r="BG109">
-        <f>IF(TRIM($Q$109)&lt;&gt;"",TRIM($Q$109),TRIM($R$109))</f>
+        <f>IF($Q$109="",$R$109,$Q$109)</f>
         <v/>
       </c>
     </row>

</xml_diff>